<commit_message>
start livestock endogenisation. Add function for excre/cap and LU per livestock type.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F59525-ADD8-4CD9-9898-43BA308FB548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37991B52-B9B2-4C23-B5BC-F99FA541E12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="2240" yWindow="2240" windowWidth="14400" windowHeight="7360" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="93">
   <si>
     <t>Scenario</t>
   </si>
@@ -186,9 +186,6 @@
     <t>Bovines heads</t>
   </si>
   <si>
-    <t>No.</t>
-  </si>
-  <si>
     <t>kgN excreted by bovines head</t>
   </si>
   <si>
@@ -300,9 +297,6 @@
     <t>Poultry % excretion in the barn as slurry</t>
   </si>
   <si>
-    <t>used as a goal but may be adjusted according to territory situation</t>
-  </si>
-  <si>
     <t>Historical trend</t>
   </si>
   <si>
@@ -315,13 +309,13 @@
     <t>if the territory requested is not found in the data, the business as usual column will be blank and you have to define all variables.</t>
   </si>
   <si>
-    <t>Taken ad the last historical value. Used as a goal but may be adjusted according to territory situation</t>
-  </si>
-  <si>
-    <t>No. Ou prop</t>
-  </si>
-  <si>
-    <t>endogeneiser la demande carnée totale</t>
+    <t>Animal nitrogen net import</t>
+  </si>
+  <si>
+    <t>Historical trend. Used as a goal but may be adjusted according to territory situation</t>
+  </si>
+  <si>
+    <t>LU</t>
   </si>
 </sst>
 </file>
@@ -711,7 +705,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
@@ -767,7 +761,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7366DC0-2904-4121-B11A-C21AC0D88D02}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.08984375" customWidth="1"/>
@@ -800,7 +794,7 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -811,7 +805,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -855,7 +849,7 @@
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -866,7 +860,7 @@
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -877,7 +871,7 @@
         <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -888,78 +882,18 @@
         <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" t="s">
-        <v>49</v>
-      </c>
-      <c r="E14" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
-      </c>
-      <c r="E15" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" t="s">
-        <v>49</v>
-      </c>
-      <c r="E16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -992,12 +926,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2581441D-9B75-4E72-BCEB-BD35B582F9B5}">
   <sheetPr codeName="Feuil4"/>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.36328125" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="3" max="3" width="4.54296875" customWidth="1"/>
+    <col min="4" max="4" width="6.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -1063,73 +998,73 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" t="s">
         <v>50</v>
       </c>
-      <c r="B6" t="s">
-        <v>51</v>
-      </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
@@ -1140,7 +1075,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -1151,7 +1086,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
@@ -1162,7 +1097,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
@@ -1173,7 +1108,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
@@ -1184,7 +1119,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1195,7 +1130,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
@@ -1206,7 +1141,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
@@ -1217,7 +1152,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -1228,7 +1163,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1239,7 +1174,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -1250,7 +1185,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1261,7 +1196,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1272,7 +1207,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1283,7 +1218,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1294,7 +1229,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -1305,7 +1240,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -1316,7 +1251,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -1327,7 +1262,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -1338,7 +1273,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -1349,7 +1284,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -1360,7 +1295,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -1371,7 +1306,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -1382,7 +1317,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -1393,7 +1328,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -1404,7 +1339,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -1415,7 +1350,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
@@ -1426,7 +1361,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
@@ -1437,7 +1372,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
@@ -1448,13 +1383,79 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B41" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" t="s">
+        <v>92</v>
+      </c>
+      <c r="E42" t="s">
         <v>86</v>
       </c>
-      <c r="B41" t="s">
-        <v>14</v>
-      </c>
-      <c r="E41" t="s">
-        <v>33</v>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" t="s">
+        <v>92</v>
+      </c>
+      <c r="E43" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>92</v>
+      </c>
+      <c r="E44" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>92</v>
+      </c>
+      <c r="E45" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>92</v>
+      </c>
+      <c r="E46" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>92</v>
+      </c>
+      <c r="E47" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add extrapolation functions, completed Livestock stuffs
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37991B52-B9B2-4C23-B5BC-F99FA541E12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418DE415-222B-4E38-8062-E8FC624E29F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2240" yWindow="2240" windowWidth="14400" windowHeight="7360" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="95">
   <si>
     <t>Scenario</t>
   </si>
@@ -165,27 +165,6 @@
     <t xml:space="preserve">Total nitrogen net import </t>
   </si>
   <si>
-    <t>Feed nitrogen net import</t>
-  </si>
-  <si>
-    <t>Caprines heads</t>
-  </si>
-  <si>
-    <t>Equines heads</t>
-  </si>
-  <si>
-    <t>Porcines heads</t>
-  </si>
-  <si>
-    <t>Poultry heads</t>
-  </si>
-  <si>
-    <t>Ovines heads</t>
-  </si>
-  <si>
-    <t>Bovines heads</t>
-  </si>
-  <si>
     <t>kgN excreted by bovines head</t>
   </si>
   <si>
@@ -309,13 +288,40 @@
     <t>if the territory requested is not found in the data, the business as usual column will be blank and you have to define all variables.</t>
   </si>
   <si>
-    <t>Animal nitrogen net import</t>
-  </si>
-  <si>
     <t>Historical trend. Used as a goal but may be adjusted according to territory situation</t>
   </si>
   <si>
     <t>LU</t>
+  </si>
+  <si>
+    <t>Total LU</t>
+  </si>
+  <si>
+    <t>Historical trend, see prop for each livestock in technical sheet</t>
+  </si>
+  <si>
+    <t>prop</t>
+  </si>
+  <si>
+    <t>Bovines LU</t>
+  </si>
+  <si>
+    <t>Ovines LU</t>
+  </si>
+  <si>
+    <t>Caprines LU</t>
+  </si>
+  <si>
+    <t>Equines LU</t>
+  </si>
+  <si>
+    <t>Porcines LU</t>
+  </si>
+  <si>
+    <t>Poultry LU</t>
+  </si>
+  <si>
+    <t>Logistic</t>
   </si>
 </sst>
 </file>
@@ -705,7 +711,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
@@ -761,7 +767,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7366DC0-2904-4121-B11A-C21AC0D88D02}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.08984375" customWidth="1"/>
@@ -794,7 +800,7 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -805,7 +811,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -849,7 +855,7 @@
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -860,7 +866,7 @@
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -871,33 +877,23 @@
         <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="E10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -931,8 +927,8 @@
   <cols>
     <col min="1" max="1" width="42.36328125" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="4.54296875" customWidth="1"/>
-    <col min="4" max="4" width="6.08984375" customWidth="1"/>
+    <col min="3" max="3" width="17.26953125" customWidth="1"/>
+    <col min="4" max="4" width="12.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -998,73 +994,73 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
@@ -1075,7 +1071,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -1086,7 +1082,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
@@ -1097,7 +1093,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
@@ -1108,7 +1104,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
@@ -1119,7 +1115,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1130,7 +1126,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
@@ -1141,7 +1137,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
@@ -1152,7 +1148,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -1163,7 +1159,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1174,7 +1170,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -1185,7 +1181,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1196,7 +1192,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1207,7 +1203,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1218,7 +1214,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1229,7 +1225,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -1240,7 +1236,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -1251,7 +1247,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -1262,7 +1258,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -1273,7 +1269,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -1284,7 +1280,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -1295,7 +1291,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -1306,7 +1302,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -1317,7 +1313,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -1328,7 +1324,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -1339,7 +1335,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -1350,7 +1346,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
@@ -1361,7 +1357,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
@@ -1372,7 +1368,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
@@ -1383,7 +1379,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
         <v>14</v>
@@ -1394,68 +1390,68 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="B42" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E42" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E43" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E44" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>91</v>
       </c>
       <c r="B45" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E45" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="B46" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E46" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>93</v>
       </c>
       <c r="B47" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E47" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add final prospective for business as usual. Add proportion of each crops.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418DE415-222B-4E38-8062-E8FC624E29F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F28985F-BDC3-445C-8151-276A1C61FE48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="94">
   <si>
     <t>Scenario</t>
   </si>
@@ -111,9 +111,6 @@
     <t>Edible animal per capita protein ingestion (excl fish)</t>
   </si>
   <si>
-    <t>Grassland area</t>
-  </si>
-  <si>
     <t>Arable area</t>
   </si>
   <si>
@@ -144,9 +141,6 @@
     <t>culture</t>
   </si>
   <si>
-    <t>area change</t>
-  </si>
-  <si>
     <t>Surface change tab is used to give general indication of crop rotation. This will give specific surface constraint for the model.</t>
   </si>
   <si>
@@ -162,9 +156,6 @@
     <t>You can enforce the given values by adding TRUE in the enforce column. Caution, if the sum of the enforced area is beyond total surface area, you will get an error.</t>
   </si>
   <si>
-    <t xml:space="preserve">Total nitrogen net import </t>
-  </si>
-  <si>
     <t>kgN excreted by bovines head</t>
   </si>
   <si>
@@ -282,9 +273,6 @@
     <t>INSEE data</t>
   </si>
   <si>
-    <t>Computed from urban population</t>
-  </si>
-  <si>
     <t>if the territory requested is not found in the data, the business as usual column will be blank and you have to define all variables.</t>
   </si>
   <si>
@@ -322,6 +310,15 @@
   </si>
   <si>
     <t>Logistic</t>
+  </si>
+  <si>
+    <t>Net import of vegetal pdcts</t>
+  </si>
+  <si>
+    <t>Permanent grassland area</t>
+  </si>
+  <si>
+    <t>area proportion (%)</t>
   </si>
 </sst>
 </file>
@@ -711,27 +708,27 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
@@ -800,7 +797,7 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -811,7 +808,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -822,7 +819,7 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -833,7 +830,7 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -844,51 +841,51 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>91</v>
       </c>
       <c r="B9" t="s">
         <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E10" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -902,16 +899,19 @@
   <sheetPr codeName="Feuil3"/>
   <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="20.453125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="C1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -945,513 +945,513 @@
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E11" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
       </c>
       <c r="E14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
       </c>
       <c r="E15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
       </c>
       <c r="E16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
       </c>
       <c r="E17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
       </c>
       <c r="E21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
       </c>
       <c r="E23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
       </c>
       <c r="E24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
       </c>
       <c r="E25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
       </c>
       <c r="E26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
       </c>
       <c r="E27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
       </c>
       <c r="E28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
       </c>
       <c r="E29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
       </c>
       <c r="E31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
       </c>
       <c r="E32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
       </c>
       <c r="E33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
       </c>
       <c r="E34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
       </c>
       <c r="E35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
       </c>
       <c r="E36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
       </c>
       <c r="E37" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
       </c>
       <c r="E38" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
       </c>
       <c r="E39" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
       </c>
       <c r="E40" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B41" t="s">
         <v>14</v>
       </c>
       <c r="E41" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B42" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E42" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B43" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E43" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B44" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E44" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B45" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E45" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B46" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E46" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E47" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add a new class ton compute Ymax for each culture in each region. Completed...
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F28985F-BDC3-445C-8151-276A1C61FE48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F59900-B301-4A72-AB8D-C48598885423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="95">
   <si>
     <t>Scenario</t>
   </si>
@@ -319,6 +319,9 @@
   </si>
   <si>
     <t>area proportion (%)</t>
+  </si>
+  <si>
+    <t>Y_max</t>
   </si>
 </sst>
 </file>
@@ -897,13 +900,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67912879-D449-4AD5-BD69-7447EF2F4940}">
   <sheetPr codeName="Feuil3"/>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="20.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -912,6 +915,9 @@
       </c>
       <c r="C1" t="s">
         <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add scenar data for Livestock productivity
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F59900-B301-4A72-AB8D-C48598885423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85285D45-2F1B-49C5-BFD4-A569C06C671B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="107">
   <si>
     <t>Scenario</t>
   </si>
@@ -321,7 +321,43 @@
     <t>area proportion (%)</t>
   </si>
   <si>
-    <t>Y_max</t>
+    <t>Bovines productivity</t>
+  </si>
+  <si>
+    <t>Ovines productivity</t>
+  </si>
+  <si>
+    <t>Caprines productivity</t>
+  </si>
+  <si>
+    <t>Equines productivity</t>
+  </si>
+  <si>
+    <t>Porcines productivity</t>
+  </si>
+  <si>
+    <t>Poultry productivity</t>
+  </si>
+  <si>
+    <t>kgcarcass/LU</t>
+  </si>
+  <si>
+    <t>Bovines dairy productivity</t>
+  </si>
+  <si>
+    <t>Poultry dairy productivity</t>
+  </si>
+  <si>
+    <t>kg/LU</t>
+  </si>
+  <si>
+    <t>Ovines and Caprines dairy productivity</t>
+  </si>
+  <si>
+    <t>Ymax (kgN/ha)</t>
+  </si>
+  <si>
+    <t>k (kgN/ha)</t>
   </si>
 </sst>
 </file>
@@ -900,13 +936,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67912879-D449-4AD5-BD69-7447EF2F4940}">
   <sheetPr codeName="Feuil3"/>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="20.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -917,7 +953,10 @@
         <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>105</v>
+      </c>
+      <c r="E1" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -928,7 +967,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2581441D-9B75-4E72-BCEB-BD35B582F9B5}">
   <sheetPr codeName="Feuil4"/>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.36328125" customWidth="1"/>
@@ -1460,6 +1499,105 @@
         <v>32</v>
       </c>
     </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" t="s">
+        <v>100</v>
+      </c>
+      <c r="E48" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>95</v>
+      </c>
+      <c r="B49" t="s">
+        <v>100</v>
+      </c>
+      <c r="E49" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>96</v>
+      </c>
+      <c r="B50" t="s">
+        <v>100</v>
+      </c>
+      <c r="E50" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" t="s">
+        <v>100</v>
+      </c>
+      <c r="E51" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" t="s">
+        <v>100</v>
+      </c>
+      <c r="E52" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>99</v>
+      </c>
+      <c r="B53" t="s">
+        <v>100</v>
+      </c>
+      <c r="E53" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>101</v>
+      </c>
+      <c r="B54" t="s">
+        <v>103</v>
+      </c>
+      <c r="E54" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" t="s">
+        <v>103</v>
+      </c>
+      <c r="E55" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>102</v>
+      </c>
+      <c r="B56" t="s">
+        <v>103</v>
+      </c>
+      <c r="E56" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Splitted caprines and ovines dairy productivity.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3D6DF1-1577-43AD-9D23-9BD7A4CCE7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221A8DB3-0EDB-4DE9-A45D-00AEB8153370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-7575" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="109">
   <si>
     <t>Scenario</t>
   </si>
@@ -162,9 +162,6 @@
     <t>Bovines % excretion on grassland</t>
   </si>
   <si>
-    <t>Bovines % excretion in the barn</t>
-  </si>
-  <si>
     <t>Bovines % excretion in the barn as litter manure</t>
   </si>
   <si>
@@ -177,9 +174,6 @@
     <t>Ovines % excretion on grassland</t>
   </si>
   <si>
-    <t>Ovines % excretion in the barn</t>
-  </si>
-  <si>
     <t>Ovines % excretion in the barn as litter manure</t>
   </si>
   <si>
@@ -192,9 +186,6 @@
     <t>Equines % excretion on grassland</t>
   </si>
   <si>
-    <t>Equines % excretion in the barn</t>
-  </si>
-  <si>
     <t>Equines % excretion in the barn as litter manure</t>
   </si>
   <si>
@@ -207,9 +198,6 @@
     <t>Caprines % excretion on grassland</t>
   </si>
   <si>
-    <t>Caprines % excretion in the barn</t>
-  </si>
-  <si>
     <t>Caprines % excretion in the barn as litter manure</t>
   </si>
   <si>
@@ -222,9 +210,6 @@
     <t>Porcines % excretion on grassland</t>
   </si>
   <si>
-    <t>Porcines % excretion in the barn</t>
-  </si>
-  <si>
     <t>Porcines % excretion in the barn as litter manure</t>
   </si>
   <si>
@@ -237,9 +222,6 @@
     <t>Poultry % excretion on grassland</t>
   </si>
   <si>
-    <t>Poultry % excretion in the barn</t>
-  </si>
-  <si>
     <t>Poultry % excretion in the barn as litter manure</t>
   </si>
   <si>
@@ -351,9 +333,6 @@
     <t>Weight import/export balance</t>
   </si>
   <si>
-    <t>Weight area</t>
-  </si>
-  <si>
     <t>Ovines dairy productivity</t>
   </si>
   <si>
@@ -376,6 +355,15 @@
   </si>
   <si>
     <t>kgN excreted by poultry LU</t>
+  </si>
+  <si>
+    <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+  </si>
+  <si>
+    <t>NH3 volatilization coefficient for synthetic nitrogen</t>
+  </si>
+  <si>
+    <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
   </si>
 </sst>
 </file>
@@ -765,7 +753,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
@@ -854,7 +842,7 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -865,7 +853,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -909,40 +897,40 @@
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B9" t="s">
         <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -987,16 +975,16 @@
         <v>33</v>
       </c>
       <c r="B1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C1" t="s">
         <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1007,7 +995,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2581441D-9B75-4E72-BCEB-BD35B582F9B5}">
   <sheetPr codeName="Feuil4"/>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.36328125" customWidth="1"/>
@@ -1035,51 +1023,51 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -1090,7 +1078,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -1104,81 +1092,81 @@
         <v>108</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
         <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="B10" t="s">
         <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>105</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
@@ -1189,7 +1177,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
@@ -1200,7 +1188,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1211,7 +1199,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
@@ -1222,7 +1210,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
@@ -1233,7 +1221,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -1244,7 +1232,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1255,7 +1243,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -1266,7 +1254,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1277,7 +1265,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1288,7 +1276,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1299,7 +1287,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1310,7 +1298,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -1321,7 +1309,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -1332,7 +1320,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -1343,7 +1331,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -1354,7 +1342,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -1365,7 +1353,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -1376,7 +1364,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -1387,7 +1375,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -1398,7 +1386,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -1409,7 +1397,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -1420,7 +1408,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -1431,7 +1419,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
@@ -1442,10 +1430,10 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B39" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E39" t="s">
         <v>32</v>
@@ -1453,10 +1441,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B40" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E40" t="s">
         <v>32</v>
@@ -1464,10 +1452,10 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E41" t="s">
         <v>32</v>
@@ -1475,10 +1463,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E42" t="s">
         <v>32</v>
@@ -1486,10 +1474,10 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E43" t="s">
         <v>32</v>
@@ -1497,10 +1485,10 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B44" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E44" t="s">
         <v>32</v>
@@ -1508,68 +1496,68 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B45" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="E45" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B46" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="E46" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B47" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="E47" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B48" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="E48" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B49" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="E49" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
+        <v>87</v>
+      </c>
+      <c r="B50" t="s">
         <v>88</v>
       </c>
-      <c r="B50" t="s">
-        <v>94</v>
-      </c>
       <c r="E50" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
@@ -1577,98 +1565,43 @@
         <v>89</v>
       </c>
       <c r="B51" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E51" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B52" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E52" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
+        <v>99</v>
+      </c>
+      <c r="B53" t="s">
         <v>91</v>
       </c>
-      <c r="B53" t="s">
-        <v>94</v>
-      </c>
       <c r="E53" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B54" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E54" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>93</v>
-      </c>
-      <c r="B55" t="s">
-        <v>94</v>
-      </c>
-      <c r="E55" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>95</v>
-      </c>
-      <c r="B56" t="s">
-        <v>97</v>
-      </c>
-      <c r="E56" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>105</v>
-      </c>
-      <c r="B57" t="s">
-        <v>97</v>
-      </c>
-      <c r="E57" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
         <v>106</v>
-      </c>
-      <c r="B58" t="s">
-        <v>97</v>
-      </c>
-      <c r="E58" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>96</v>
-      </c>
-      <c r="B59" t="s">
-        <v>97</v>
-      </c>
-      <c r="E59" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added file for exponential production function. Add small fix to manage absence of line Function production in Scenario.xlsx. Started to update prospective class
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882AD981-C2A8-4366-B833-9194631E4174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8331B8-F24A-4FBA-BBD1-E6BB76580524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-7575" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="110">
   <si>
     <t>Scenario</t>
   </si>
@@ -364,6 +364,9 @@
   </si>
   <si>
     <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
+  </si>
+  <si>
+    <t>Production function</t>
   </si>
 </sst>
 </file>
@@ -730,7 +733,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6FCCA24-34E1-444C-AF4C-91646ADAA8F7}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.54296875" customWidth="1"/>
@@ -799,6 +802,11 @@
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Error located and corrected. Added an excel_dict to locate lines where to get...
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882AD981-C2A8-4366-B833-9194631E4174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8331B8-F24A-4FBA-BBD1-E6BB76580524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-7575" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="110">
   <si>
     <t>Scenario</t>
   </si>
@@ -364,6 +364,9 @@
   </si>
   <si>
     <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
+  </si>
+  <si>
+    <t>Production function</t>
   </si>
 </sst>
 </file>
@@ -730,7 +733,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6FCCA24-34E1-444C-AF4C-91646ADAA8F7}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.54296875" customWidth="1"/>
@@ -799,6 +802,11 @@
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modification of scenario.xslx to include new stuff about import/export and methanisation.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8331B8-F24A-4FBA-BBD1-E6BB76580524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A73269F-F3AE-4BFB-AF59-8B631245255A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="116">
   <si>
     <t>Scenario</t>
   </si>
@@ -240,9 +240,6 @@
     <t>if the territory requested is not found in the data, the business as usual column will be blank and you have to define all variables.</t>
   </si>
   <si>
-    <t>Historical trend. Used as a goal but may be adjusted according to territory situation</t>
-  </si>
-  <si>
     <t>LU</t>
   </si>
   <si>
@@ -276,9 +273,6 @@
     <t>Logistic</t>
   </si>
   <si>
-    <t>Net import of vegetal pdcts</t>
-  </si>
-  <si>
     <t>Permanent grassland area</t>
   </si>
   <si>
@@ -330,9 +324,6 @@
     <t>Weight synthetic fertilizer use</t>
   </si>
   <si>
-    <t>Weight import/export balance</t>
-  </si>
-  <si>
     <t>Ovines dairy productivity</t>
   </si>
   <si>
@@ -367,6 +358,33 @@
   </si>
   <si>
     <t>Production function</t>
+  </si>
+  <si>
+    <t>Import of vegetal pdcts</t>
+  </si>
+  <si>
+    <t>Export of vegetal pdcts</t>
+  </si>
+  <si>
+    <t>Methanisation</t>
+  </si>
+  <si>
+    <t>GWh</t>
+  </si>
+  <si>
+    <t>2006 data. Used as a goal but may be adjusted according to territory situation</t>
+  </si>
+  <si>
+    <t>2021 data. Used as a goal but may be adjusted according to territory situation</t>
+  </si>
+  <si>
+    <t>Weight import</t>
+  </si>
+  <si>
+    <t>Weight export</t>
+  </si>
+  <si>
+    <t>Weight energy</t>
   </si>
 </sst>
 </file>
@@ -806,7 +824,7 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -817,7 +835,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7366DC0-2904-4121-B11A-C21AC0D88D02}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.08984375" customWidth="1"/>
@@ -861,7 +879,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -910,7 +928,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -921,46 +939,68 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="B9" t="s">
         <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>108</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
         <v>29</v>
       </c>
       <c r="E12" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E14" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -983,16 +1023,16 @@
         <v>33</v>
       </c>
       <c r="B1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C1" t="s">
         <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1003,7 +1043,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2581441D-9B75-4E72-BCEB-BD35B582F9B5}">
   <sheetPr codeName="Feuil4"/>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.36328125" customWidth="1"/>
@@ -1031,62 +1071,62 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
+        <v>114</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
+        <v>115</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -1097,7 +1137,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>108</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
@@ -1108,29 +1148,29 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
@@ -1141,7 +1181,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
@@ -1152,7 +1192,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
@@ -1163,7 +1203,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B14" t="s">
         <v>39</v>
@@ -1174,29 +1214,29 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>101</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1207,7 +1247,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
@@ -1218,7 +1258,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
@@ -1229,7 +1269,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -1240,7 +1280,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1251,7 +1291,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -1262,7 +1302,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1273,7 +1313,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1284,7 +1324,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1295,7 +1335,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1306,7 +1346,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -1317,7 +1357,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -1328,7 +1368,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -1339,7 +1379,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -1350,7 +1390,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -1361,7 +1401,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -1372,7 +1412,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -1383,7 +1423,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -1394,7 +1434,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -1405,7 +1445,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -1416,7 +1456,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -1427,7 +1467,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
@@ -1438,10 +1478,10 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B39" t="s">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="E39" t="s">
         <v>32</v>
@@ -1449,10 +1489,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B40" t="s">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="E40" t="s">
         <v>32</v>
@@ -1460,10 +1500,10 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E41" t="s">
         <v>32</v>
@@ -1471,10 +1511,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E42" t="s">
         <v>32</v>
@@ -1482,10 +1522,10 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E43" t="s">
         <v>32</v>
@@ -1493,10 +1533,10 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E44" t="s">
         <v>32</v>
@@ -1504,112 +1544,134 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E45" t="s">
-        <v>106</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B46" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E46" t="s">
-        <v>106</v>
+        <v>32</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E47" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B48" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E48" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>82</v>
+      </c>
+      <c r="B49" t="s">
         <v>86</v>
       </c>
-      <c r="B49" t="s">
-        <v>88</v>
-      </c>
       <c r="E49" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B50" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E50" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E51" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E52" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="B53" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E53" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E54" t="s">
-        <v>106</v>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" t="s">
+        <v>89</v>
+      </c>
+      <c r="E55" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>88</v>
+      </c>
+      <c r="B56" t="s">
+        <v>89</v>
+      </c>
+      <c r="E56" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated all files scenario files for all production function to add a Energy production goal and a weight for energy production.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A73269F-F3AE-4BFB-AF59-8B631245255A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4626E19-E102-4985-ACED-D637B132CB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
modification of scenario.xlsx file to add methanizer
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4626E19-E102-4985-ACED-D637B132CB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86E25A9-7A05-489B-995E-9A50511276F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-3312" yWindow="-17388" windowWidth="30936" windowHeight="16896" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -93,9 +93,6 @@
     <t>comment</t>
   </si>
   <si>
-    <t>ktN</t>
-  </si>
-  <si>
     <t>Urban population</t>
   </si>
   <si>
@@ -366,16 +363,13 @@
     <t>Export of vegetal pdcts</t>
   </si>
   <si>
-    <t>Methanisation</t>
-  </si>
-  <si>
-    <t>GWh</t>
-  </si>
-  <si>
     <t>2006 data. Used as a goal but may be adjusted according to territory situation</t>
   </si>
   <si>
-    <t>2021 data. Used as a goal but may be adjusted according to territory situation</t>
+    <t>GWh/yr</t>
+  </si>
+  <si>
+    <t>ktN/yr</t>
   </si>
   <si>
     <t>Weight import</t>
@@ -385,6 +379,12 @@
   </si>
   <si>
     <t>Weight energy</t>
+  </si>
+  <si>
+    <t>Regional 2021 data mapped on 2006 33 region plant production. Used as a goal but may be adjusted according to territory situation</t>
+  </si>
+  <si>
+    <t>Methaniser production</t>
   </si>
 </sst>
 </file>
@@ -774,27 +774,27 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
@@ -824,7 +824,7 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -868,139 +868,139 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>110</v>
       </c>
       <c r="E9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" t="s">
         <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
         <v>68</v>
-      </c>
-      <c r="B11" t="s">
-        <v>67</v>
-      </c>
-      <c r="E11" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" t="s">
         <v>109</v>
       </c>
-      <c r="B14" t="s">
-        <v>110</v>
-      </c>
       <c r="E14" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1020,19 +1020,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" t="s">
         <v>90</v>
-      </c>
-      <c r="E1" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1066,612 +1066,612 @@
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2">
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
       </c>
       <c r="E17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
       </c>
       <c r="E20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
       </c>
       <c r="E21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
       </c>
       <c r="E23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
       </c>
       <c r="E24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
       </c>
       <c r="E25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
       </c>
       <c r="E27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
       </c>
       <c r="E28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
       </c>
       <c r="E30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
       </c>
       <c r="E31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
       </c>
       <c r="E32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
       </c>
       <c r="E33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
       </c>
       <c r="E34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
       </c>
       <c r="E35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
       </c>
       <c r="E36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
       </c>
       <c r="E37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
       </c>
       <c r="E38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
       </c>
       <c r="E39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
       </c>
       <c r="E40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E42" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E43" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E44" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B46" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E46" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B47" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E47" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B48" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B49" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E49" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B50" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E50" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B51" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E51" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
+        <v>84</v>
+      </c>
+      <c r="B52" t="s">
         <v>85</v>
       </c>
-      <c r="B52" t="s">
-        <v>86</v>
-      </c>
       <c r="E52" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B53" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E53" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B54" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E54" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B55" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
+        <v>87</v>
+      </c>
+      <c r="B56" t="s">
         <v>88</v>
       </c>
-      <c r="B56" t="s">
-        <v>89</v>
-      </c>
       <c r="E56" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resolve "move urban population to technical tab"
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario.xlsx
+++ b/src/grafs_e/data/scenario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD51356-E19C-40C4-B616-4338F98A40B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94237931-F45C-4B07-8A2C-E7A080464D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{EBD5F612-DF6B-4870-80D9-98AC0696C5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="doc" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="123">
   <si>
     <t>Scenario</t>
   </si>
@@ -403,6 +403,9 @@
   </si>
   <si>
     <t>2023 data. Used as a goal but may be adjusted according to territory situation</t>
+  </si>
+  <si>
+    <t>Weight methaniser input</t>
   </si>
 </sst>
 </file>
@@ -853,7 +856,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7366DC0-2904-4121-B11A-C21AC0D88D02}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.08984375" customWidth="1"/>
@@ -891,18 +894,18 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
         <v>21</v>
@@ -913,7 +916,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -924,18 +927,18 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
@@ -946,18 +949,18 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>110</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B9" t="s">
         <v>110</v>
@@ -968,29 +971,29 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="B10" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>108</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="E11" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -1001,23 +1004,12 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>114</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>114</v>
-      </c>
-      <c r="B14" t="s">
-        <v>109</v>
-      </c>
-      <c r="E14" t="s">
         <v>121</v>
       </c>
     </row>
@@ -1061,7 +1053,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2581441D-9B75-4E72-BCEB-BD35B582F9B5}">
   <sheetPr codeName="Feuil4"/>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.36328125" customWidth="1"/>
@@ -1144,29 +1136,29 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
+        <v>122</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
@@ -1177,7 +1169,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
@@ -1188,29 +1180,29 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B13" t="s">
         <v>38</v>
@@ -1221,7 +1213,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
@@ -1232,7 +1224,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B15" t="s">
         <v>38</v>
@@ -1243,7 +1235,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
         <v>38</v>
@@ -1254,29 +1246,29 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>101</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="E18" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
@@ -1287,7 +1279,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -1298,7 +1290,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1309,7 +1301,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -1320,7 +1312,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1331,7 +1323,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1342,7 +1334,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1353,7 +1345,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1364,7 +1356,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -1375,7 +1367,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -1386,7 +1378,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -1397,7 +1389,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -1408,7 +1400,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -1419,7 +1411,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -1430,7 +1422,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -1441,7 +1433,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -1452,7 +1444,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -1463,7 +1455,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -1474,7 +1466,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -1485,7 +1477,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
@@ -1496,7 +1488,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
@@ -1507,7 +1499,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
@@ -1518,10 +1510,10 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B41" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E41" t="s">
         <v>31</v>
@@ -1529,10 +1521,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B42" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E42" t="s">
         <v>31</v>
@@ -1540,7 +1532,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s">
         <v>69</v>
@@ -1551,7 +1543,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B44" t="s">
         <v>69</v>
@@ -1562,7 +1554,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B45" t="s">
         <v>69</v>
@@ -1573,7 +1565,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B46" t="s">
         <v>69</v>
@@ -1584,29 +1576,29 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B47" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="E47" t="s">
-        <v>102</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B48" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="E48" t="s">
-        <v>102</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B49" t="s">
         <v>85</v>
@@ -1617,7 +1609,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B50" t="s">
         <v>85</v>
@@ -1628,7 +1620,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B51" t="s">
         <v>85</v>
@@ -1639,7 +1631,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B52" t="s">
         <v>85</v>
@@ -1650,10 +1642,10 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B53" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E53" t="s">
         <v>102</v>
@@ -1661,10 +1653,10 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B54" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E54" t="s">
         <v>102</v>
@@ -1672,7 +1664,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B55" t="s">
         <v>88</v>
@@ -1683,7 +1675,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B56" t="s">
         <v>88</v>
@@ -1694,41 +1686,35 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="B57" t="s">
-        <v>69</v>
-      </c>
-      <c r="C57">
-        <v>0.06</v>
+        <v>88</v>
       </c>
       <c r="E57" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="B58" t="s">
-        <v>69</v>
-      </c>
-      <c r="C58">
-        <v>0.02</v>
+        <v>88</v>
       </c>
       <c r="E58" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B59" t="s">
         <v>69</v>
       </c>
       <c r="C59">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
       <c r="E59" t="s">
         <v>116</v>
@@ -1736,13 +1722,13 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B60" t="s">
         <v>69</v>
       </c>
       <c r="C60">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="E60" t="s">
         <v>116</v>
@@ -1750,15 +1736,43 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B61" t="s">
         <v>69</v>
       </c>
       <c r="C61">
+        <v>0.09</v>
+      </c>
+      <c r="E61" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>119</v>
+      </c>
+      <c r="B62" t="s">
+        <v>69</v>
+      </c>
+      <c r="C62">
+        <v>0.04</v>
+      </c>
+      <c r="E62" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>120</v>
+      </c>
+      <c r="B63" t="s">
+        <v>69</v>
+      </c>
+      <c r="C63">
         <v>0.79</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E63" t="s">
         <v>116</v>
       </c>
     </row>

</xml_diff>